<commit_message>
seeds: update alias/fluors/plasmids/rnas/tags; ui: remove legacy single-upload pages; keep unified uploaders
</commit_message>
<xml_diff>
--- a/carp_app/seed_kits/dyes_fluors_tags_fusions/tags.xlsx
+++ b/carp_app/seed_kits/dyes_fluors_tags_fusions/tags.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/carp_app/seed_kits/dyes_fluors_tags_fusions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F644FBA-E4EF-3C41-8A96-79572B3E384F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B107327-5292-A340-8967-EB404D8A637F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6920" yWindow="3860" windowWidth="27640" windowHeight="16680" xr2:uid="{89706445-C364-CF42-9B42-6F31A2F723ED}"/>
+    <workbookView xWindow="32960" yWindow="16860" windowWidth="27640" windowHeight="16680" xr2:uid="{89706445-C364-CF42-9B42-6F31A2F723ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>2Xcox8A</t>
   </si>
@@ -111,6 +111,12 @@
   </si>
   <si>
     <t>nucleus</t>
+  </si>
+  <si>
+    <t>GMN</t>
+  </si>
+  <si>
+    <t>CDT1</t>
   </si>
 </sst>
 </file>
@@ -496,7 +502,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7128CD98-9A0B-0D46-9F23-B9C08D30033B}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -593,6 +599,16 @@
         <v>23</v>
       </c>
     </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>